<commit_message>
Fix the two-way grid for replacement capex and label the cost columns
Chow's targeted fixes to workbook v5:
- The two-way grid (B120:D123) now includes the replacement driver B16, so it matches the cash-flow base when B16 is nonzero. Tested: with replacement 0.01 the grid cell at 200 bn and the cash base equals B21 (-181.31).
- Column D is the legacy total-cost ratio (0.9383, which includes D&A, financing and tax). The labels now say so: columns B and C are cash-cost cases, column D is the legacy total-cost reconciliation.

No input or base value changed: primary NPV -163.12 bn, break-even capex 30.60 bn, break-even attendance 74.0 million.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
+++ b/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
@@ -10349,14 +10349,14 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Two-way sensitivity: primary NPV pre-tax (THB bn), capital cost (rows) by cash operating-cost share (columns), ticket-only revenue, base WACC and life</t>
+          <t>Two-way sensitivity: primary NPV pre-tax (THB bn), capital cost (rows) by cost share (columns). Columns B and C are cash-cost cases; column D is the legacy total-cost reconciliation (includes D&amp;A, financing and tax). Ticket-only revenue, base WACC and life; replacement per B16.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Capital cost (THB bn), rows; cash operating-cost share, columns</t>
+          <t>Capital cost (THB bn), rows; cost share, columns (B, C cash; D legacy total-cost)</t>
         </is>
       </c>
       <c r="B119" s="3" t="n">
@@ -10376,15 +10376,15 @@
         <v>150</v>
       </c>
       <c r="B120" s="4">
-        <f>$B$15*(1-B$119)*$B$27-$A120*($B$28/$B$9)</f>
+        <f>$B$15*(1-B$119)*$B$27-$A120*($B$28/$B$9)-$B$16*$A120*$B$27</f>
         <v/>
       </c>
       <c r="C120" s="4">
-        <f>$B$15*(1-C$119)*$B$27-$A120*($B$28/$B$9)</f>
+        <f>$B$15*(1-C$119)*$B$27-$A120*($B$28/$B$9)-$B$16*$A120*$B$27</f>
         <v/>
       </c>
       <c r="D120" s="4">
-        <f>$B$15*(1-D$119)*$B$27-$A120*($B$28/$B$9)</f>
+        <f>$B$15*(1-D$119)*$B$27-$A120*($B$28/$B$9)-$B$16*$A120*$B$27</f>
         <v/>
       </c>
     </row>
@@ -10393,15 +10393,15 @@
         <v>200</v>
       </c>
       <c r="B121" s="4">
-        <f>$B$15*(1-B$119)*$B$27-$A121*($B$28/$B$9)</f>
+        <f>$B$15*(1-B$119)*$B$27-$A121*($B$28/$B$9)-$B$16*$A121*$B$27</f>
         <v/>
       </c>
       <c r="C121" s="4">
-        <f>$B$15*(1-C$119)*$B$27-$A121*($B$28/$B$9)</f>
+        <f>$B$15*(1-C$119)*$B$27-$A121*($B$28/$B$9)-$B$16*$A121*$B$27</f>
         <v/>
       </c>
       <c r="D121" s="4">
-        <f>$B$15*(1-D$119)*$B$27-$A121*($B$28/$B$9)</f>
+        <f>$B$15*(1-D$119)*$B$27-$A121*($B$28/$B$9)-$B$16*$A121*$B$27</f>
         <v/>
       </c>
     </row>
@@ -10410,15 +10410,15 @@
         <v>250</v>
       </c>
       <c r="B122" s="4">
-        <f>$B$15*(1-B$119)*$B$27-$A122*($B$28/$B$9)</f>
+        <f>$B$15*(1-B$119)*$B$27-$A122*($B$28/$B$9)-$B$16*$A122*$B$27</f>
         <v/>
       </c>
       <c r="C122" s="4">
-        <f>$B$15*(1-C$119)*$B$27-$A122*($B$28/$B$9)</f>
+        <f>$B$15*(1-C$119)*$B$27-$A122*($B$28/$B$9)-$B$16*$A122*$B$27</f>
         <v/>
       </c>
       <c r="D122" s="4">
-        <f>$B$15*(1-D$119)*$B$27-$A122*($B$28/$B$9)</f>
+        <f>$B$15*(1-D$119)*$B$27-$A122*($B$28/$B$9)-$B$16*$A122*$B$27</f>
         <v/>
       </c>
     </row>
@@ -10427,15 +10427,15 @@
         <v>300</v>
       </c>
       <c r="B123" s="4">
-        <f>$B$15*(1-B$119)*$B$27-$A123*($B$28/$B$9)</f>
+        <f>$B$15*(1-B$119)*$B$27-$A123*($B$28/$B$9)-$B$16*$A123*$B$27</f>
         <v/>
       </c>
       <c r="C123" s="4">
-        <f>$B$15*(1-C$119)*$B$27-$A123*($B$28/$B$9)</f>
+        <f>$B$15*(1-C$119)*$B$27-$A123*($B$28/$B$9)-$B$16*$A123*$B$27</f>
         <v/>
       </c>
       <c r="D123" s="4">
-        <f>$B$15*(1-D$119)*$B$27-$A123*($B$28/$B$9)</f>
+        <f>$B$15*(1-D$119)*$B$27-$A123*($B$28/$B$9)-$B$16*$A123*$B$27</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix the sensitivity chart layout: title, plot and legend no longer overlap
The sensitivity chart on the Charts sheet is taller, the plot area sits below the title, and the legend is placed below the value-axis labels. Chart data, series and formulas are unchanged.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
+++ b/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\DisneyDiD\econ-disney-seminar\seminar\workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116124F0-F692-4717-9B5D-8D334BC020D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EECB300-5F20-4148-9761-803C73EF4FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2301,11 +2301,29 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.33920117521367521"/>
+          <c:y val="1.2121212121212121E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="1"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.23303899572649572"/>
+          <c:y val="0.11515151515151516"/>
+          <c:w val="0.74859626068376073"/>
+          <c:h val="0.76363636363636367"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
@@ -2814,6 +2832,16 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.27641452991452992"/>
+          <c:y val="0.96957134335480799"/>
+          <c:w val="0.44717083333333335"/>
+          <c:h val="2.739835361488905E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="1"/>
       <c:txPr>
         <a:bodyPr/>
@@ -2950,7 +2978,7 @@
       <xdr:row>50</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="9360000" cy="7200000"/>
+    <xdr:ext cx="9360000" cy="8382000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="4" name="Chart 3">

</xml_diff>

<commit_message>
Annual cash flow chart on a log axis: capital outflow and operating inflow as separate series
The cash-flow chart on the Charts sheet uses a log axis from 1 to 1000 (decades). A log axis cannot show negative values, so the chart plots the capital outflow (absolute value, red, labelled -100.0) and the operating cash flow (positive, navy) as two series. Zero years are not plotted. Two helper columns on the Appraisal sheet (U and V, years 0 to 22) hold these values; the signed cash flow in column J is unchanged.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
+++ b/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\DisneyDiD\econ-disney-seminar\seminar\workbook\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temp\claude\C--Users-user-AppData-Roaming-Claude-scratch-workspaces-c7acaf2f-ed5f-4f26-814b-0755985b8641-704b7f5d-017e-4c68-a76d-e0c46600fd5a-scratch-2026-10-16-ee569e\885493fd-7279-48f0-8993-cb2538820dce\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EECB300-5F20-4148-9761-803C73EF4FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79AD1439-7B9B-42B1-9376-FFB27DA66F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="440">
   <si>
     <t>Parameter</t>
   </si>
@@ -1336,6 +1336,12 @@
   </si>
   <si>
     <t>Park-only operator appraisal: charts</t>
+  </si>
+  <si>
+    <t>Capital outflow, absolute (THB bn)</t>
+  </si>
+  <si>
+    <t>Operating cash flow (THB bn)</t>
   </si>
 </sst>
 </file>
@@ -1346,7 +1352,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1363,6 +1369,14 @@
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1385,7 +1399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1398,6 +1412,9 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1433,7 +1450,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1300" b="1"/>
-              <a:t>Annual cash flow before tax, park-only (THB bn)</a:t>
+              <a:t>Annual cash flow before tax, park-only (THB bn, log scale)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1452,18 +1469,18 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Appraisal!$J$40</c:f>
+              <c:f>Appraisal!$U$40</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Cash flow before tax</c:v>
+                  <c:v>Capital outflow, absolute (THB bn)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="1F3864"/>
+              <a:srgbClr val="C0504D"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -1473,7 +1490,7 @@
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
-              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:numFmt formatCode="\-#,##0.0" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
                 <a:ln>
@@ -1508,7 +1525,7 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
-              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:numFmt formatCode="\-#,##0.0" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
                 <a:ln>
@@ -1640,78 +1657,78 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Appraisal!$J$41:$J$63</c:f>
+              <c:f>Appraisal!$U$41:$U$63</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="23"/>
                 <c:pt idx="0">
-                  <c:v>-100</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-100</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.3395922101449287</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1719,6 +1736,188 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-6E58-4402-AA0C-BC86BA6AC45A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Appraisal!$V$40</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operating cash flow (THB bn)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F3864"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>Appraisal!$A$41:$A$63</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="23"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Appraisal!$V$41:$V$63</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="23"/>
+                <c:pt idx="0">
+                  <c:v>#N/A</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>#N/A</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>5.3395922101449287</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>#N/A</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D25F-44B6-B4FF-3F12DE3843DC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1731,6 +1930,7 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="60"/>
+        <c:overlap val="100"/>
         <c:axId val="10"/>
         <c:axId val="100"/>
       </c:barChart>
@@ -1762,9 +1962,10 @@
       <c:valAx>
         <c:axId val="100"/>
         <c:scaling>
+          <c:logBase val="10"/>
           <c:orientation val="minMax"/>
-          <c:max val="20"/>
-          <c:min val="-120"/>
+          <c:max val="1000"/>
+          <c:min val="1"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1807,9 +2008,13 @@
         <c:crossAx val="10"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
-        <c:majorUnit val="20"/>
+        <c:majorUnit val="10"/>
       </c:valAx>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="1"/>
@@ -5747,7 +5952,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:S135"/>
+  <dimension ref="A1:V135"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -5763,6 +5968,7 @@
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
+    <col min="21" max="22" width="18.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -6080,12 +6286,12 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" ht="29" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
         <v>339</v>
       </c>
@@ -6143,8 +6349,14 @@
       <c r="S40" s="7" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U40" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="V40" s="10" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>0</v>
       </c>
@@ -6220,8 +6432,16 @@
         <f>SUM($Q$41:Q41)</f>
         <v>-100</v>
       </c>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U41" s="5">
+        <f t="shared" ref="U41:U63" si="14">IF(J41&lt;0,-J41,NA())</f>
+        <v>100</v>
+      </c>
+      <c r="V41" s="5" t="e">
+        <f t="shared" ref="V41:V63" si="15">IF(J41&gt;0,J41,NA())</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>1</v>
       </c>
@@ -6282,7 +6502,7 @@
         <v>0</v>
       </c>
       <c r="P42" s="5">
-        <f t="shared" ref="P42:P63" si="14">MAX(0,O42-O41)</f>
+        <f t="shared" ref="P42:P63" si="16">MAX(0,O42-O41)</f>
         <v>0</v>
       </c>
       <c r="Q42" s="5">
@@ -6297,8 +6517,16 @@
         <f>SUM($Q$41:Q42)</f>
         <v>-200</v>
       </c>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U42" s="5">
+        <f t="shared" si="14"/>
+        <v>100</v>
+      </c>
+      <c r="V42" s="5" t="e">
+        <f t="shared" si="15"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>2</v>
       </c>
@@ -6359,7 +6587,7 @@
         <v>0</v>
       </c>
       <c r="P43" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q43" s="5">
@@ -6374,8 +6602,16 @@
         <f>SUM($Q$41:Q43)</f>
         <v>-194.66040778985507</v>
       </c>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U43" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V43" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>3</v>
       </c>
@@ -6436,7 +6672,7 @@
         <v>0</v>
       </c>
       <c r="P44" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q44" s="5">
@@ -6451,8 +6687,16 @@
         <f>SUM($Q$41:Q44)</f>
         <v>-189.32081557971014</v>
       </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U44" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V44" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>4</v>
       </c>
@@ -6513,7 +6757,7 @@
         <v>0</v>
       </c>
       <c r="P45" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q45" s="5">
@@ -6528,8 +6772,16 @@
         <f>SUM($Q$41:Q45)</f>
         <v>-183.98122336956521</v>
       </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U45" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V45" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>5</v>
       </c>
@@ -6590,7 +6842,7 @@
         <v>0</v>
       </c>
       <c r="P46" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q46" s="5">
@@ -6605,8 +6857,16 @@
         <f>SUM($Q$41:Q46)</f>
         <v>-178.64163115942029</v>
       </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U46" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V46" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>6</v>
       </c>
@@ -6667,7 +6927,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q47" s="5">
@@ -6682,8 +6942,16 @@
         <f>SUM($Q$41:Q47)</f>
         <v>-173.30203894927536</v>
       </c>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U47" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V47" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>7</v>
       </c>
@@ -6744,7 +7012,7 @@
         <v>0</v>
       </c>
       <c r="P48" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q48" s="5">
@@ -6759,8 +7027,16 @@
         <f>SUM($Q$41:Q48)</f>
         <v>-167.96244673913043</v>
       </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U48" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V48" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>8</v>
       </c>
@@ -6821,7 +7097,7 @@
         <v>0</v>
       </c>
       <c r="P49" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q49" s="5">
@@ -6836,8 +7112,16 @@
         <f>SUM($Q$41:Q49)</f>
         <v>-162.6228545289855</v>
       </c>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U49" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V49" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>9</v>
       </c>
@@ -6898,7 +7182,7 @@
         <v>0</v>
       </c>
       <c r="P50" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q50" s="5">
@@ -6913,8 +7197,16 @@
         <f>SUM($Q$41:Q50)</f>
         <v>-157.28326231884057</v>
       </c>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U50" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V50" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>10</v>
       </c>
@@ -6975,7 +7267,7 @@
         <v>0</v>
       </c>
       <c r="P51" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q51" s="5">
@@ -6990,8 +7282,16 @@
         <f>SUM($Q$41:Q51)</f>
         <v>-151.94367010869564</v>
       </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U51" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V51" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>11</v>
       </c>
@@ -7052,7 +7352,7 @@
         <v>0</v>
       </c>
       <c r="P52" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q52" s="5">
@@ -7067,8 +7367,16 @@
         <f>SUM($Q$41:Q52)</f>
         <v>-146.60407789855071</v>
       </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U52" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V52" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>12</v>
       </c>
@@ -7129,7 +7437,7 @@
         <v>0</v>
       </c>
       <c r="P53" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q53" s="5">
@@ -7144,8 +7452,16 @@
         <f>SUM($Q$41:Q53)</f>
         <v>-141.26448568840578</v>
       </c>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U53" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V53" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>13</v>
       </c>
@@ -7206,7 +7522,7 @@
         <v>0</v>
       </c>
       <c r="P54" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q54" s="5">
@@ -7221,8 +7537,16 @@
         <f>SUM($Q$41:Q54)</f>
         <v>-135.92489347826086</v>
       </c>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U54" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V54" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>14</v>
       </c>
@@ -7283,7 +7607,7 @@
         <v>0</v>
       </c>
       <c r="P55" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q55" s="5">
@@ -7298,8 +7622,16 @@
         <f>SUM($Q$41:Q55)</f>
         <v>-130.58530126811593</v>
       </c>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U55" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V55" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>15</v>
       </c>
@@ -7360,7 +7692,7 @@
         <v>0</v>
       </c>
       <c r="P56" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q56" s="5">
@@ -7375,8 +7707,16 @@
         <f>SUM($Q$41:Q56)</f>
         <v>-125.245709057971</v>
       </c>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U56" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V56" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>16</v>
       </c>
@@ -7437,7 +7777,7 @@
         <v>0</v>
       </c>
       <c r="P57" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q57" s="5">
@@ -7452,8 +7792,16 @@
         <f>SUM($Q$41:Q57)</f>
         <v>-119.90611684782607</v>
       </c>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U57" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V57" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>17</v>
       </c>
@@ -7514,7 +7862,7 @@
         <v>0</v>
       </c>
       <c r="P58" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q58" s="5">
@@ -7529,8 +7877,16 @@
         <f>SUM($Q$41:Q58)</f>
         <v>-114.56652463768114</v>
       </c>
-    </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U58" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V58" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>18</v>
       </c>
@@ -7591,7 +7947,7 @@
         <v>0</v>
       </c>
       <c r="P59" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q59" s="5">
@@ -7606,8 +7962,16 @@
         <f>SUM($Q$41:Q59)</f>
         <v>-109.22693242753621</v>
       </c>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U59" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V59" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>19</v>
       </c>
@@ -7668,7 +8032,7 @@
         <v>0</v>
       </c>
       <c r="P60" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q60" s="5">
@@ -7683,8 +8047,16 @@
         <f>SUM($Q$41:Q60)</f>
         <v>-103.88734021739128</v>
       </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U60" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V60" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>20</v>
       </c>
@@ -7745,7 +8117,7 @@
         <v>0</v>
       </c>
       <c r="P61" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q61" s="5">
@@ -7760,8 +8132,16 @@
         <f>SUM($Q$41:Q61)</f>
         <v>-98.547748007246355</v>
       </c>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U61" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V61" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>21</v>
       </c>
@@ -7822,7 +8202,7 @@
         <v>0</v>
       </c>
       <c r="P62" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q62" s="5">
@@ -7837,8 +8217,16 @@
         <f>SUM($Q$41:Q62)</f>
         <v>-93.208155797101426</v>
       </c>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="U62" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V62" s="5">
+        <f t="shared" si="15"/>
+        <v>5.3395922101449287</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>22</v>
       </c>
@@ -7899,7 +8287,7 @@
         <v>0</v>
       </c>
       <c r="P63" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="Q63" s="5">
@@ -7914,6 +8302,14 @@
         <f>SUM($Q$41:Q63)</f>
         <v>-93.208155797101426</v>
       </c>
+      <c r="U63" s="5" t="e">
+        <f t="shared" si="14"/>
+        <v>#N/A</v>
+      </c>
+      <c r="V63" s="5" t="e">
+        <f t="shared" si="15"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
@@ -7981,35 +8377,35 @@
         <v>0</v>
       </c>
       <c r="F68" s="4">
-        <f t="shared" ref="F68:F94" si="15">SUMPRODUCT($B$41:$B$63*($A$41:$A$63&gt;=$B$8+E68)*($A$41:$A$63&lt;$B$8+E68+$B$7))</f>
+        <f t="shared" ref="F68:F94" si="17">SUMPRODUCT($B$41:$B$63*($A$41:$A$63&gt;=$B$8+E68)*($A$41:$A$63&lt;$B$8+E68+$B$7))</f>
         <v>9.0908772291197089</v>
       </c>
       <c r="G68" s="5">
-        <f t="shared" ref="G68:G94" si="16">(D68-C68*$B$5)*$B$15*F68-B68*$B$28-I68*B68*$B$9*F68</f>
+        <f t="shared" ref="G68:G94" si="18">(D68-C68*$B$5)*$B$15*F68-B68*$B$28-I68*B68*$B$9*F68</f>
         <v>-144.05101535660108</v>
       </c>
       <c r="H68" s="5">
-        <f t="shared" ref="H68:H94" si="17">(D68-C68*$B$5)*$C$15*F68-B68*($C$9/$B$9)*$B$28-I68*B68*$C$9*F68</f>
+        <f t="shared" ref="H68:H94" si="19">(D68-C68*$B$5)*$C$15*F68-B68*($C$9/$B$9)*$B$28-I68*B68*$C$9*F68</f>
         <v>-259.41977774562076</v>
       </c>
       <c r="I68" s="4">
-        <f t="shared" ref="I68:I93" si="18">$B$16</f>
+        <f t="shared" ref="I68:I93" si="20">$B$16</f>
         <v>0</v>
       </c>
       <c r="J68" s="5">
-        <f t="shared" ref="J68:J94" si="19">D68*$B$15-C68*$B$5*$B$15-B68*$B$9/$B$18</f>
+        <f t="shared" ref="J68:J94" si="21">D68*$B$15-C68*$B$5*$B$15-B68*$B$9/$B$18</f>
         <v>-4.6604077898550713</v>
       </c>
       <c r="K68" s="5">
-        <f t="shared" ref="K68:K94" si="20">IF($B$18&lt;$B$7,"n/a",G68-$B$17*MAX(0,J68)*F68)</f>
+        <f t="shared" ref="K68:K94" si="22">IF($B$18&lt;$B$7,"n/a",G68-$B$17*MAX(0,J68)*F68)</f>
         <v>-144.05101535660108</v>
       </c>
       <c r="L68" s="5">
-        <f t="shared" ref="L68:L94" si="21">D68*$C$15-C68*$B$5*$C$15-B68*$C$9/$C$18</f>
+        <f t="shared" ref="L68:L94" si="23">D68*$C$15-C68*$B$5*$C$15-B68*$C$9/$C$18</f>
         <v>-11.758386413043478</v>
       </c>
       <c r="M68" s="5">
-        <f t="shared" ref="M68:M94" si="22">IF($C$18&lt;$C$7,"n/a",H68-$B$17*MAX(0,L68)*F68)</f>
+        <f t="shared" ref="M68:M94" si="24">IF($C$18&lt;$C$7,"n/a",H68-$B$17*MAX(0,L68)*F68)</f>
         <v>-259.41977774562076</v>
       </c>
       <c r="N68" t="s">
@@ -8033,35 +8429,35 @@
         <v>0</v>
       </c>
       <c r="F69" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G69" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-153.68064498623073</v>
       </c>
       <c r="H69" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-273.86422219006528</v>
       </c>
       <c r="I69" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J69" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-5.1604077898550713</v>
       </c>
       <c r="K69" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-153.68064498623073</v>
       </c>
       <c r="L69" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-12.508386413043478</v>
       </c>
       <c r="M69" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-273.86422219006528</v>
       </c>
       <c r="N69" t="s">
@@ -8085,35 +8481,35 @@
         <v>0</v>
       </c>
       <c r="F70" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G70" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-134.42138572697144</v>
       </c>
       <c r="H70" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-244.97533330117631</v>
       </c>
       <c r="I70" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J70" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-4.1604077898550713</v>
       </c>
       <c r="K70" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-134.42138572697144</v>
       </c>
       <c r="L70" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-11.008386413043478</v>
       </c>
       <c r="M70" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-244.97533330117631</v>
       </c>
       <c r="N70" t="s">
@@ -8137,35 +8533,35 @@
         <v>0</v>
       </c>
       <c r="F71" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G71" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-163.31027461586035</v>
       </c>
       <c r="H71" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-288.30866663450968</v>
       </c>
       <c r="I71" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J71" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-5.6604077898550731</v>
       </c>
       <c r="K71" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-163.31027461586035</v>
       </c>
       <c r="L71" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-13.258386413043478</v>
       </c>
       <c r="M71" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-288.30866663450968</v>
       </c>
       <c r="N71" t="s">
@@ -8189,35 +8585,35 @@
         <v>0</v>
       </c>
       <c r="F72" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G72" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-124.79175609734182</v>
       </c>
       <c r="H72" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-230.53088885673191</v>
       </c>
       <c r="I72" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J72" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-3.6604077898550713</v>
       </c>
       <c r="K72" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-124.79175609734182</v>
       </c>
       <c r="L72" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-10.258386413043478</v>
       </c>
       <c r="M72" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-230.53088885673191</v>
       </c>
       <c r="N72" t="s">
@@ -8241,35 +8637,35 @@
         <v>0</v>
       </c>
       <c r="F73" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G73" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-182.56953387511959</v>
       </c>
       <c r="H73" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-317.19755552339853</v>
       </c>
       <c r="I73" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J73" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-6.6604077898550713</v>
       </c>
       <c r="K73" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-182.56953387511959</v>
       </c>
       <c r="L73" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-14.758386413043478</v>
       </c>
       <c r="M73" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-317.19755552339853</v>
       </c>
       <c r="N73" t="s">
@@ -8293,35 +8689,35 @@
         <v>0</v>
       </c>
       <c r="F74" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G74" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-105.53249683808258</v>
       </c>
       <c r="H74" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-201.64199996784305</v>
       </c>
       <c r="I74" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J74" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-2.6604077898550713</v>
       </c>
       <c r="K74" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-105.53249683808258</v>
       </c>
       <c r="L74" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-8.7583864130434783</v>
       </c>
       <c r="M74" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-201.64199996784305</v>
       </c>
       <c r="N74" t="s">
@@ -8345,35 +8741,35 @@
         <v>0</v>
       </c>
       <c r="F75" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G75" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-152.2327970400431</v>
       </c>
       <c r="H75" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-264.38685643379603</v>
       </c>
       <c r="I75" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J75" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-5.5604069293478275</v>
       </c>
       <c r="K75" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-152.2327970400431</v>
       </c>
       <c r="L75" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-12.304766983695652</v>
       </c>
       <c r="M75" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-264.38685643379603</v>
       </c>
       <c r="N75" t="s">
@@ -8397,35 +8793,35 @@
         <v>0</v>
       </c>
       <c r="F76" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G76" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-135.86923367315907</v>
       </c>
       <c r="H76" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-254.45269905744547</v>
       </c>
       <c r="I76" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J76" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-3.7604086503623186</v>
       </c>
       <c r="K76" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-135.86923367315907</v>
       </c>
       <c r="L76" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-11.212005842391305</v>
       </c>
       <c r="M76" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-254.45269905744547</v>
       </c>
       <c r="N76" t="s">
@@ -8449,35 +8845,35 @@
         <v>0</v>
       </c>
       <c r="F77" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G77" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-160.41457872348511</v>
       </c>
       <c r="H77" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-269.35393512197129</v>
       </c>
       <c r="I77" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J77" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-6.4604060688405802</v>
       </c>
       <c r="K77" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-160.41457872348511</v>
       </c>
       <c r="L77" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-12.851147554347827</v>
       </c>
       <c r="M77" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-269.35393512197129</v>
       </c>
       <c r="N77" t="s">
@@ -8501,35 +8897,35 @@
         <v>0</v>
       </c>
       <c r="F78" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G78" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-127.68745198971706</v>
       </c>
       <c r="H78" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-249.48562036927018</v>
       </c>
       <c r="I78" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J78" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-2.860409510869566</v>
       </c>
       <c r="K78" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-127.68745198971706</v>
       </c>
       <c r="L78" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-10.665625271739129</v>
       </c>
       <c r="M78" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-249.48562036927018</v>
       </c>
       <c r="N78" t="s">
@@ -8553,35 +8949,35 @@
         <v>0</v>
       </c>
       <c r="F79" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G79" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-176.7781420903691</v>
       </c>
       <c r="H79" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-279.28809249832187</v>
       </c>
       <c r="I79" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J79" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-8.2604043478260856</v>
       </c>
       <c r="K79" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-176.7781420903691</v>
       </c>
       <c r="L79" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-13.943908695652173</v>
       </c>
       <c r="M79" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-279.28809249832187</v>
       </c>
       <c r="N79" t="s">
@@ -8605,35 +9001,35 @@
         <v>0</v>
       </c>
       <c r="F80" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G80" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-111.32388862283307</v>
       </c>
       <c r="H80" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-239.55146299291965</v>
       </c>
       <c r="I80" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J80" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.0604112318840588</v>
       </c>
       <c r="K80" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-111.32388862283307</v>
       </c>
       <c r="L80" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-9.5728641304347821</v>
       </c>
       <c r="M80" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-239.55146299291965</v>
       </c>
       <c r="N80" t="s">
@@ -8657,35 +9053,35 @@
         <v>0</v>
       </c>
       <c r="F81" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G81" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-133.4421548113595</v>
       </c>
       <c r="H81" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-252.97924350028205</v>
       </c>
       <c r="I81" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J81" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-3.4934290398550694</v>
       </c>
       <c r="K81" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-133.4421548113595</v>
       </c>
       <c r="L81" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-11.049925163043477</v>
       </c>
       <c r="M81" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-252.97924350028205</v>
       </c>
       <c r="N81" t="s">
@@ -8709,35 +9105,35 @@
         <v>0</v>
       </c>
       <c r="F82" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G82" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-154.65987590184267</v>
       </c>
       <c r="H82" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-265.86031199095942</v>
       </c>
       <c r="I82" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J82" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-5.8273865398550733</v>
       </c>
       <c r="K82" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-154.65987590184267</v>
       </c>
       <c r="L82" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-12.466847663043479</v>
       </c>
       <c r="M82" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-265.86031199095942</v>
       </c>
       <c r="N82" t="s">
@@ -8761,35 +9157,35 @@
         <v>0</v>
       </c>
       <c r="F83" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G83" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-122.83329426611789</v>
       </c>
       <c r="H83" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-246.53870925494337</v>
       </c>
       <c r="I83" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J83" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-2.3264502898550674</v>
       </c>
       <c r="K83" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-122.83329426611789</v>
       </c>
       <c r="L83" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-10.341463913043476</v>
       </c>
       <c r="M83" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-246.53870925494337</v>
       </c>
       <c r="N83" t="s">
@@ -8813,35 +9209,35 @@
         <v>0</v>
       </c>
       <c r="F84" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G84" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-165.26873644708425</v>
       </c>
       <c r="H84" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-272.30084623629813</v>
       </c>
       <c r="I84" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J84" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-6.9943652898550717</v>
       </c>
       <c r="K84" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-165.26873644708425</v>
       </c>
       <c r="L84" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-13.175308913043478</v>
       </c>
       <c r="M84" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-272.30084623629813</v>
       </c>
       <c r="N84" t="s">
@@ -8865,35 +9261,35 @@
         <v>0</v>
       </c>
       <c r="F85" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G85" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-101.61557317563475</v>
       </c>
       <c r="H85" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-233.65764076426601</v>
       </c>
       <c r="I85" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J85" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>7.5072101449293882E-3</v>
       </c>
       <c r="K85" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-101.6292226007869</v>
       </c>
       <c r="L85" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-8.9245414130434799</v>
       </c>
       <c r="M85" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-233.65764076426601</v>
       </c>
       <c r="N85" t="s">
@@ -8917,35 +9313,35 @@
         <v>0</v>
       </c>
       <c r="F86" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G86" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-186.48645753756739</v>
       </c>
       <c r="H86" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-285.18191472697549</v>
       </c>
       <c r="I86" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J86" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-9.328322789855072</v>
       </c>
       <c r="K86" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-186.48645753756739</v>
       </c>
       <c r="L86" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-14.592231413043478</v>
       </c>
       <c r="M86" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-285.18191472697549</v>
       </c>
       <c r="N86" t="s">
@@ -8969,35 +9365,35 @@
         <v>0</v>
       </c>
       <c r="F87" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G87" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-164.28950553147232</v>
       </c>
       <c r="H87" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-280.30475643540393</v>
       </c>
       <c r="I87" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J87" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-6.3273865398550733</v>
       </c>
       <c r="K87" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-164.28950553147232</v>
       </c>
       <c r="L87" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-13.216847663043479</v>
       </c>
       <c r="M87" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-280.30475643540393</v>
       </c>
       <c r="N87" t="s">
@@ -9021,35 +9417,35 @@
         <v>0</v>
       </c>
       <c r="F88" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G88" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-123.81252518172984</v>
       </c>
       <c r="H88" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-238.5347990558376</v>
       </c>
       <c r="I88" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J88" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-2.9934290398550694</v>
       </c>
       <c r="K88" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-123.81252518172984</v>
       </c>
       <c r="L88" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-10.299925163043477</v>
       </c>
       <c r="M88" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-238.5347990558376</v>
       </c>
       <c r="N88" t="s">
@@ -9073,35 +9469,35 @@
         <v>0</v>
       </c>
       <c r="F89" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G89" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-184.52799570634352</v>
       </c>
       <c r="H89" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-301.18973512518704</v>
       </c>
       <c r="I89" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J89" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-7.9943652898550734</v>
       </c>
       <c r="K89" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-184.52799570634352</v>
       </c>
       <c r="L89" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-14.675308913043478</v>
       </c>
       <c r="M89" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-301.18973512518704</v>
       </c>
       <c r="N89" t="s">
@@ -9125,35 +9521,35 @@
         <v>0</v>
       </c>
       <c r="F90" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G90" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-103.57403500685862</v>
       </c>
       <c r="H90" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-217.64982036605451</v>
       </c>
       <c r="I90" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J90" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.3264502898550674</v>
       </c>
       <c r="K90" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-103.57403500685862</v>
       </c>
       <c r="L90" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-8.8414639130434765</v>
       </c>
       <c r="M90" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-217.64982036605451</v>
       </c>
       <c r="N90" t="s">
@@ -9177,35 +9573,35 @@
         <v>0</v>
       </c>
       <c r="F91" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G91" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-225.00497605608589</v>
       </c>
       <c r="H91" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-342.95969250475326</v>
       </c>
       <c r="I91" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J91" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-11.328322789855072</v>
       </c>
       <c r="K91" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-225.00497605608589</v>
       </c>
       <c r="L91" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-17.592231413043478</v>
       </c>
       <c r="M91" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-342.95969250475326</v>
       </c>
       <c r="N91" t="s">
@@ -9229,35 +9625,35 @@
         <v>0</v>
       </c>
       <c r="F92" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G92" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-63.097054657116246</v>
       </c>
       <c r="H92" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-175.87986298648829</v>
       </c>
       <c r="I92" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J92" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>2.0075072101449294</v>
       </c>
       <c r="K92" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-66.747054973916278</v>
       </c>
       <c r="L92" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-5.9245414130434799</v>
       </c>
       <c r="M92" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-175.87986298648829</v>
       </c>
       <c r="N92" t="s">
@@ -9281,35 +9677,35 @@
         <v>1</v>
       </c>
       <c r="F93" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8.4174789158515821</v>
       </c>
       <c r="G93" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-147.64668774445229</v>
       </c>
       <c r="H93" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-261.60267486734432</v>
       </c>
       <c r="I93" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J93" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-4.6604077898550713</v>
       </c>
       <c r="K93" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-147.64668774445229</v>
       </c>
       <c r="L93" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-11.758386413043478</v>
       </c>
       <c r="M93" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-261.60267486734432</v>
       </c>
       <c r="N93" t="s">
@@ -9333,15 +9729,15 @@
         <v>0</v>
       </c>
       <c r="F94" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.0908772291197089</v>
       </c>
       <c r="G94" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>-287.85647706968189</v>
       </c>
       <c r="H94" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>-475.12797031524201</v>
       </c>
       <c r="I94" s="4">
@@ -9349,19 +9745,19 @@
         <v>7.9093281148075664E-2</v>
       </c>
       <c r="J94" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-4.6604077898550713</v>
       </c>
       <c r="K94" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>-287.85647706968189</v>
       </c>
       <c r="L94" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-11.758386413043478</v>
       </c>
       <c r="M94" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-475.12797031524201</v>
       </c>
       <c r="N94" t="s">
@@ -9427,15 +9823,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G103" s="4">
-        <f t="shared" ref="G103:G113" si="23">(1+B103)^(-$B$8)*(1-(1+B103)^(-C103))/(1-1/(1+B103))</f>
+        <f t="shared" ref="G103:G113" si="25">(1+B103)^(-$B$8)*(1-(1+B103)^(-C103))/(1-1/(1+B103))</f>
         <v>9.0908772291197018</v>
       </c>
       <c r="H103" s="5">
-        <f t="shared" ref="H103:H113" si="24">($B$9/$B$8)*(1-(1+B103)^(-$B$8))/(1-1/(1+B103))</f>
+        <f t="shared" ref="H103:H113" si="26">($B$9/$B$8)*(1-(1+B103)^(-$B$8))/(1-1/(1+B103))</f>
         <v>192.59259259259238</v>
       </c>
       <c r="I103" s="5">
-        <f t="shared" ref="I103:I113" si="25">(F103*(1-$B$5)-E103*$B$9)*G103-H103</f>
+        <f t="shared" ref="I103:I113" si="27">(F103*(1-$B$5)-E103*$B$9)*G103-H103</f>
         <v>-144.05101535660091</v>
       </c>
     </row>
@@ -9463,15 +9859,15 @@
         <v>14.169225000000003</v>
       </c>
       <c r="G104" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>9.0908772291197018</v>
       </c>
       <c r="H104" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>192.59259259259238</v>
       </c>
       <c r="I104" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-163.12348144932429</v>
       </c>
     </row>
@@ -9487,7 +9883,7 @@
         <v>30</v>
       </c>
       <c r="D105">
-        <f t="shared" ref="D105:D111" si="26">$B$19</f>
+        <f t="shared" ref="D105:D111" si="28">$B$19</f>
         <v>1</v>
       </c>
       <c r="E105" s="4">
@@ -9499,15 +9895,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G105" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>10.423873465858767</v>
       </c>
       <c r="H105" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>192.59259259259238</v>
       </c>
       <c r="I105" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-136.93335903475651</v>
       </c>
     </row>
@@ -9523,7 +9919,7 @@
         <v>40</v>
       </c>
       <c r="D106">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
       <c r="E106" s="4">
@@ -9535,15 +9931,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G106" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>11.041308642357691</v>
       </c>
       <c r="H106" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>192.59259259259238</v>
       </c>
       <c r="I106" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-133.6365069760534</v>
       </c>
     </row>
@@ -9559,7 +9955,7 @@
         <v>20</v>
       </c>
       <c r="D107">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
       <c r="E107" s="4">
@@ -9571,15 +9967,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G107" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>10.820680394872868</v>
       </c>
       <c r="H107" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>194.33962264150929</v>
       </c>
       <c r="I107" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-136.5616018965782</v>
       </c>
     </row>
@@ -9595,7 +9991,7 @@
         <v>20</v>
       </c>
       <c r="D108">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
       <c r="E108" s="4">
@@ -9607,15 +10003,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G108" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>9.9009478930057568</v>
       </c>
       <c r="H108" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>193.45794392523374</v>
       </c>
       <c r="I108" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-140.59091968268936</v>
       </c>
     </row>
@@ -9631,7 +10027,7 @@
         <v>20</v>
       </c>
       <c r="D109">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
       <c r="E109" s="4">
@@ -9643,15 +10039,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G109" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>7.7396033815986929</v>
       </c>
       <c r="H109" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>190.90909090909093</v>
       </c>
       <c r="I109" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-149.58276498309522</v>
       </c>
     </row>
@@ -9668,7 +10064,7 @@
         <v>20</v>
       </c>
       <c r="D110">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
       <c r="E110" s="4">
@@ -9680,15 +10076,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G110" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>9.0908772291197018</v>
       </c>
       <c r="H110" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>192.59259259259238</v>
       </c>
       <c r="I110" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-287.85647706968166</v>
       </c>
     </row>
@@ -9704,7 +10100,7 @@
         <v>30</v>
       </c>
       <c r="D111">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
       <c r="E111" s="4">
@@ -9716,15 +10112,15 @@
         <v>23.339575000000004</v>
       </c>
       <c r="G111" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>10.423873465858767</v>
       </c>
       <c r="H111" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>192.59259259259238</v>
       </c>
       <c r="I111" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-301.82502997218319</v>
       </c>
     </row>
@@ -9752,15 +10148,15 @@
         <v>14.169225000000003</v>
       </c>
       <c r="G112" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>9.0908772291197018</v>
       </c>
       <c r="H112" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>192.59259259259238</v>
       </c>
       <c r="I112" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-306.92894316240506</v>
       </c>
     </row>
@@ -9787,15 +10183,15 @@
         <v>14.169225000000003</v>
       </c>
       <c r="G113" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>10.423873465858767</v>
       </c>
       <c r="H113" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>192.59259259259238</v>
       </c>
       <c r="I113" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>-323.69409367437572</v>
       </c>
     </row>
@@ -9825,15 +10221,15 @@
         <v>150</v>
       </c>
       <c r="B120" s="5">
-        <f t="shared" ref="B120:D123" si="27">$B$15*(1-B$119)*$B$27-$A120*($B$28/$B$9)-$B$16*$A120*$B$27</f>
+        <f t="shared" ref="B120:D123" si="29">$B$15*(1-B$119)*$B$27-$A120*($B$28/$B$9)-$B$16*$A120*$B$27</f>
         <v>-80.791281172994928</v>
       </c>
       <c r="C120" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-95.902867208452932</v>
       </c>
       <c r="D120" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-131.35311053161632</v>
       </c>
     </row>
@@ -9842,15 +10238,15 @@
         <v>200</v>
       </c>
       <c r="B121" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-128.93942932114308</v>
       </c>
       <c r="C121" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-144.05101535660108</v>
       </c>
       <c r="D121" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-179.50125867976448</v>
       </c>
     </row>
@@ -9859,15 +10255,15 @@
         <v>250</v>
       </c>
       <c r="B122" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-177.08757746929123</v>
       </c>
       <c r="C122" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-192.19916350474924</v>
       </c>
       <c r="D122" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-227.64940682791263</v>
       </c>
     </row>
@@ -9876,15 +10272,15 @@
         <v>300</v>
       </c>
       <c r="B123" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-225.23572561743936</v>
       </c>
       <c r="C123" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-240.34731165289736</v>
       </c>
       <c r="D123" s="5">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>-275.79755497606072</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add payback rows to the Appraisal sheet
Rows 33 to 37 give the payback for the park-only case (column B) and the 300 bn complex reference (column C):
- Cumulative cash flow over the operating life, before tax.
- Years of operation needed for nominal payback, and the estimated payback year from the start of construction.
- Whether nominal payback falls within the operating life.
- Estimated discounted payback year at WACC, which reads "never" when the present value of the margin never covers the present value of the capital cost.

Results: park-only nominal payback about year 39 (37.5 operating years), complex about year 95; neither pays back at 8 percent. Checked against a year-by-year calculation on a higher-ticket variant.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
+++ b/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temp\claude\C--Users-user-AppData-Roaming-Claude-scratch-workspaces-c7acaf2f-ed5f-4f26-814b-0755985b8641-704b7f5d-017e-4c68-a76d-e0c46600fd5a-scratch-2026-10-16-ee569e\885493fd-7279-48f0-8993-cb2538820dce\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE231D8-B9DB-4A00-8EF5-2DA226AA4BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E680D22-5C87-486E-9428-8E01C66D3393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="445">
   <si>
     <t>Parameter</t>
   </si>
@@ -1342,15 +1342,31 @@
   </si>
   <si>
     <t>Operating cash flow (THB bn)</t>
+  </si>
+  <si>
+    <t>Cumulative cash flow over the operating life, before tax (THB bn)</t>
+  </si>
+  <si>
+    <t>Years of operation needed for nominal payback</t>
+  </si>
+  <si>
+    <t>Estimated nominal payback year (from start of construction)</t>
+  </si>
+  <si>
+    <t>Nominal payback within the operating life</t>
+  </si>
+  <si>
+    <t>Estimated discounted payback year at WACC (from start of construction)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -1406,7 +1422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1423,6 +1439,16 @@
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6533,6 +6559,71 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A33" s="15" t="s">
+        <v>440</v>
+      </c>
+      <c r="B33" s="12">
+        <f>SUM(J41:J63)</f>
+        <v>-93.208155797101426</v>
+      </c>
+      <c r="C33" s="12">
+        <f>(C15*(1-C5)-C16*C9)*B7-C9</f>
+        <v>-235.16772826086958</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A34" s="15" t="s">
+        <v>441</v>
+      </c>
+      <c r="B34" s="13">
+        <f>IF(B15*(1-B5)-B16*B9&lt;=0,"never",B9/(B15*(1-B5)-B16*B9))</f>
+        <v>37.456043856684623</v>
+      </c>
+      <c r="C34" s="13">
+        <f>IF(C15*(1-C5)-C16*C9&lt;=0,"never",C9/(C15*(1-C5)-C16*C9))</f>
+        <v>92.546502521808364</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A35" s="15" t="s">
+        <v>442</v>
+      </c>
+      <c r="B35" s="13">
+        <f>IF(ISNUMBER(B34),B8+B34,"never")</f>
+        <v>39.456043856684623</v>
+      </c>
+      <c r="C35" s="13">
+        <f>IF(ISNUMBER(C34),C8+C34,"never")</f>
+        <v>94.546502521808364</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A36" s="15" t="s">
+        <v>443</v>
+      </c>
+      <c r="B36" s="14" t="str">
+        <f>IF(ISNUMBER(B34),IF(B34&lt;=B7,"Yes","No"),"No")</f>
+        <v>No</v>
+      </c>
+      <c r="C36" s="14" t="str">
+        <f>IF(ISNUMBER(C34),IF(C34&lt;=C7,"Yes","No"),"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A37" s="15" t="s">
+        <v>444</v>
+      </c>
+      <c r="B37" s="13" t="str">
+        <f>IF(B15*(1-B5)-B16*B9&lt;=0,"never",IF(B28*B6*(1+B6)^(B8-1)/(B15*(1-B5)-B16*B9)&gt;=1,"never",B8-LN(1-B28*B6*(1+B6)^(B8-1)/(B15*(1-B5)-B16*B9))/LN(1+B6)))</f>
+        <v>never</v>
+      </c>
+      <c r="C37" s="13" t="str">
+        <f>IF(C15*(1-C5)-C16*C9&lt;=0,"never",IF((C9/B9)*B28*C6*(1+C6)^(C8-1)/(C15*(1-C5)-C16*C9)&gt;=1,"never",C8-LN(1-(C9/B9)*B28*C6*(1+C6)^(C8-1)/(C15*(1-C5)-C16*C9))/LN(1+C6)))</f>
+        <v>never</v>
+      </c>
+    </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>338</v>

</xml_diff>

<commit_message>
Show value labels on the sensitivity chart bars
Both series on the sensitivity chart now show their values at the outer end of each bar (7 pt Times New Roman, one decimal). Values and formulas are unchanged.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
+++ b/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temp\claude\C--Users-user-AppData-Roaming-Claude-scratch-workspaces-c7acaf2f-ed5f-4f26-814b-0755985b8641-704b7f5d-017e-4c68-a76d-e0c46600fd5a-scratch-2026-10-16-ee569e\885493fd-7279-48f0-8993-cb2538820dce\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E680D22-5C87-486E-9428-8E01C66D3393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F8D39A-960E-47E5-B79E-1AB96DC013C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1422,7 +1422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1448,7 +1448,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2752,6 +2751,46 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="700">
+                    <a:solidFill>
+                      <a:srgbClr val="404040"/>
+                    </a:solidFill>
+                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Appraisal!$N$68:$N$94</c:f>
@@ -2960,6 +2999,46 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="700">
+                    <a:solidFill>
+                      <a:srgbClr val="404040"/>
+                    </a:solidFill>
+                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Appraisal!$N$68:$N$94</c:f>
@@ -6560,7 +6639,7 @@
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="2" t="s">
         <v>440</v>
       </c>
       <c r="B33" s="12">
@@ -6573,7 +6652,7 @@
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A34" s="15" t="s">
+      <c r="A34" s="2" t="s">
         <v>441</v>
       </c>
       <c r="B34" s="13">
@@ -6586,7 +6665,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="2" t="s">
         <v>442</v>
       </c>
       <c r="B35" s="13">
@@ -6599,7 +6678,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A36" s="15" t="s">
+      <c r="A36" s="2" t="s">
         <v>443</v>
       </c>
       <c r="B36" s="14" t="str">
@@ -6612,7 +6691,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A37" s="15" t="s">
+      <c r="A37" s="2" t="s">
         <v>444</v>
       </c>
       <c r="B37" s="13" t="str">

</xml_diff>

<commit_message>
Label the operating cash-flow bars in the annual chart
The annual cash-flow chart labelled only the two capital bars. Add value
labels to the operating bars for years 2 to 21 (5.3 THB bn each, 8 pt,
Times New Roman, outside end). Year 22 stays an empty category: the
20-year operating life from year 2 ends at year 21, so year 22 is zero by
the model rule and is not plotted.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
+++ b/seminar/workbook/Phase1_financial_appraisal_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temp\claude\C--Users-user-AppData-Roaming-Claude-scratch-workspaces-c7acaf2f-ed5f-4f26-814b-0755985b8641-704b7f5d-017e-4c68-a76d-e0c46600fd5a-scratch-2026-10-16-ee569e\885493fd-7279-48f0-8993-cb2538820dce\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94E7F13-21F4-4103-B9F9-F8F90C4DA915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{508BAA86-9B43-4AD2-9502-D3077BD120C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1802,6 +1802,886 @@
             </a:solidFill>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="8"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="9"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="10"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="11"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="12"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="13"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="14"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000C-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="15"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000D-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="16"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000E-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="17"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000F-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="18"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000010-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="19"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000011-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="20"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000012-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="21"/>
+              <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="800">
+                      <a:solidFill>
+                        <a:srgbClr val="404040"/>
+                      </a:solidFill>
+                      <a:latin typeface="Times New Roman"/>
+                      <a:ea typeface="Times New Roman"/>
+                      <a:cs typeface="Times New Roman"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000013-C1E0-44CC-9963-210863B94866}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Appraisal!$A$41:$A$63</c:f>

</xml_diff>